<commit_message>
Checked no of invalid login attempts
</commit_message>
<xml_diff>
--- a/testcases/Selected_Test_Cases.xlsx
+++ b/testcases/Selected_Test_Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c2e55e60e09c4bc/Documents/codeX/AutomationProjectsSeleniumJava/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\LiveAutomation-SeleniumJava\testcases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_2843F99744FB926409F97B1F3D59FD4ED6F1B1AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CF175D2-A925-4714-AFB5-FBBFB7A437CA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDC1218-5BD6-44BF-AA80-DBBB52751204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13500" yWindow="0" windowWidth="9636" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Selected Test Cases" sheetId="2" r:id="rId1"/>
@@ -1082,7 +1082,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1100,8 +1100,15 @@
       <sz val="9"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1138,6 +1145,12 @@
         <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1163,10 +1176,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1195,8 +1209,15 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="40% - Accent3" xfId="1" builtinId="39"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1778,74 +1799,74 @@
       <c r="M7" s="3"/>
     </row>
     <row r="8" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="5"/>
-      <c r="K8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L8" s="4"/>
-      <c r="M8" s="5"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="10"/>
+      <c r="M8" s="11"/>
     </row>
     <row r="9" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="J9" s="5"/>
-      <c r="K9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="5"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L9" s="10"/>
+      <c r="M9" s="11"/>
     </row>
     <row r="10" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -2303,74 +2324,74 @@
       <c r="M22" s="5"/>
     </row>
     <row r="23" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="I23" s="7" t="s">
+      <c r="I23" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="J23" s="7"/>
-      <c r="K23" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L23" s="6"/>
-      <c r="M23" s="7"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L23" s="10"/>
+      <c r="M23" s="11"/>
     </row>
     <row r="24" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="H24" s="7" t="s">
+      <c r="H24" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I24" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="J24" s="7"/>
-      <c r="K24" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="L24" s="6"/>
-      <c r="M24" s="7"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L24" s="10"/>
+      <c r="M24" s="11"/>
     </row>
     <row r="25" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">

</xml_diff>